<commit_message>
feat(data): synchronize exact verified project areas across index cards, map placemarks, filter attributes, and Excel registry
</commit_message>
<xml_diff>
--- a/РЕЕСТР_ПРОЕКТОВ_FERRO_DESIGN.xlsx
+++ b/РЕЕСТР_ПРОЕКТОВ_FERRO_DESIGN.xlsx
@@ -33,12 +33,6 @@
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00856404"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <sz val="10"/>
     </font>
     <font>
@@ -46,8 +40,14 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="002E7D32"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -62,14 +62,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF3CD"/>
-        <bgColor rgb="00FFF3CD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFDF0"/>
-        <bgColor rgb="00FFFDF0"/>
+        <fgColor rgb="00E8F5E9"/>
+        <bgColor rgb="00E8F5E9"/>
       </patternFill>
     </fill>
   </fills>
@@ -104,16 +98,16 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -485,19 +479,19 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="25" customWidth="1" min="9" max="9"/>
     <col width="31" customWidth="1" min="10" max="10"/>
     <col width="45" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>№</t>
@@ -520,17 +514,17 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Текущая площадь на сайте (м²)</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>ТОЧНАЯ ПЛОЩАДЬ (УТОЧНИТЬ С ЗАКАЗЧИКОМ)</t>
+          <t>Площадь (м²)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Статус верификации</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Статус объекта</t>
+          <t>Статус реализации</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -555,786 +549,858 @@
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="3" t="n">
+      <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>ЖК «Макаровский»</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Екатеринбург</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Жилая квартира</t>
         </is>
       </c>
-      <c r="E2" s="3" t="n">
-        <v>140</v>
-      </c>
-      <c r="F2" s="5" t="inlineStr"/>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="E2" s="4" t="n">
+        <v>102</v>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Подтверждено заказчиком</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Реализован</t>
         </is>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="H2" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>MAKAROVSKI_PORTUGALIA</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>project-makarovsky.html</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>Эталонный кейс с ночным рендером и комнатами</t>
         </is>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>ЖК «На Некрасова»</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Екатеринбург</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Жилая квартира</t>
         </is>
       </c>
-      <c r="E3" s="3" t="n">
-        <v>120</v>
-      </c>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="E3" s="4" t="n">
+        <v>110</v>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Подтверждено заказчиком</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>В реализации</t>
         </is>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="H3" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>NA_NEKRASOVA</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>project-nekrasova.html</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>Рендеры переименованы по комнатам</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="3" t="n">
+      <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>ЖК «Екатерининский парк»</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Екатеринбург</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Жилая квартира</t>
         </is>
       </c>
-      <c r="E4" s="3" t="n">
-        <v>110</v>
-      </c>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="E4" s="4" t="n">
+        <v>78</v>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Подтверждено заказчиком</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Проект</t>
         </is>
       </c>
-      <c r="H4" s="3" t="n">
+      <c r="H4" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>EKATER_PARK</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>project-ekater-park.html</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr"/>
+      <c r="K4" s="3" t="inlineStr"/>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>ЖК «Suomen Ranta»</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Екатеринбург</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Жилая квартира</t>
         </is>
       </c>
-      <c r="E5" s="3" t="n">
-        <v>85</v>
-      </c>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="E5" s="4" t="n">
+        <v>58</v>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Подтверждено заказчиком</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Реализован</t>
         </is>
       </c>
-      <c r="H5" s="3" t="n">
+      <c r="H5" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>SUOMEN</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>project-suomen.html</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr"/>
+      <c r="K5" s="3" t="inlineStr"/>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Отель «Номерной фонд»</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Екатеринбург</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Коммерческий объект</t>
         </is>
       </c>
-      <c r="E6" s="3" t="n">
-        <v>45</v>
-      </c>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="E6" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Подтверждено заказчиком</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Реализован</t>
         </is>
       </c>
-      <c r="H6" s="3" t="n">
+      <c r="H6" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>NOMER_OTEL</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>project-nomer-otel.html</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr"/>
+      <c r="K6" s="3" t="inlineStr"/>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Апартаменты ArtU 40 м²</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Екатеринбург</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Жилая квартира</t>
         </is>
       </c>
-      <c r="E7" s="3" t="n">
+      <c r="E7" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Подтверждено заказчиком</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Реализован</t>
         </is>
       </c>
-      <c r="H7" s="3" t="n">
+      <c r="H7" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>ARTU_40M2</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>project-artu-40m2.html</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr"/>
+      <c r="K7" s="3" t="inlineStr"/>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="3" t="n">
+      <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Гастропаб в Нижнем Тагиле</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Нижний Тагил</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Коммерческий объект</t>
         </is>
       </c>
-      <c r="E8" s="3" t="n">
-        <v>210</v>
-      </c>
-      <c r="F8" s="5" t="inlineStr"/>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="E8" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Подтверждено заказчиком</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Реализован</t>
         </is>
       </c>
-      <c r="H8" s="3" t="n">
+      <c r="H8" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>PUB_TAGIL</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>project-pub-tagil.html</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr"/>
+      <c r="K8" s="3" t="inlineStr"/>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Квартира на ГГМ</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Дом на ГГМ</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Нижний Тагил</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Жилая квартира</t>
         </is>
       </c>
-      <c r="E9" s="3" t="n">
-        <v>78</v>
-      </c>
-      <c r="F9" s="5" t="inlineStr"/>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="E9" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Подтверждено заказчиком</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Реализован</t>
         </is>
       </c>
-      <c r="H9" s="3" t="n">
+      <c r="H9" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>KRIS_GGM</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="J9" s="3" t="inlineStr">
         <is>
           <t>project-kris-ggm.html</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr"/>
+      <c r="K9" s="3" t="inlineStr"/>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="3" t="n">
+      <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Коттедж в Фатеево</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Свердловская обл.</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Загородный дом</t>
         </is>
       </c>
-      <c r="E10" s="3" t="n">
-        <v>260</v>
-      </c>
-      <c r="F10" s="5" t="inlineStr"/>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="E10" s="4" t="n">
+        <v>152</v>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Подтверждено заказчиком</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Реализован</t>
         </is>
       </c>
-      <c r="H10" s="3" t="n">
+      <c r="H10" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>ANDR_FATEEVO</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="J10" s="3" t="inlineStr">
         <is>
           <t>project-andr-fateevo.html</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr"/>
+      <c r="K10" s="3" t="inlineStr"/>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Дом в Горбуново</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Горбуново</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>Загородный дом</t>
         </is>
       </c>
-      <c r="E11" s="3" t="n">
-        <v>220</v>
-      </c>
-      <c r="F11" s="5" t="inlineStr"/>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="E11" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Подтверждено заказчиком</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Проект</t>
         </is>
       </c>
-      <c r="H11" s="3" t="n">
+      <c r="H11" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>GORBUNOVO_2FL</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="J11" s="3" t="inlineStr">
         <is>
           <t>project-gorbunovo-2fl.html</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr"/>
+      <c r="K11" s="3" t="inlineStr"/>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="3" t="n">
+      <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Комплекс A-Frame домов</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Свердловская обл.</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>Загородный дом</t>
         </is>
       </c>
-      <c r="E12" s="3" t="n">
+      <c r="E12" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Подтверждено заказчиком</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Реализован</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>A_FRAMES</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>project-a-frames.html</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Банный СПА-комплекс</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Свердловская обл.</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Коммерческий объект</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Подтверждено заказчиком</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Реализован</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>BANNIY_KOMPL</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>project-banniy-kompl.html</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Частная резиденция ХМАО</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Сургут / ХМАО</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Загородный дом</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Подтверждено заказчиком</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Проект</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>HMAO</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>project-hmao.html</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Апартаменты в Сочи</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Сочи</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Жилая квартира</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Подтверждено заказчиком</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Реализован</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>SOCHI_KVARTIRA</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>project-sochi-kvartira.html</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Квартира Данил Нагорный</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Свердловская обл.</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Загородный дом</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>96</v>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Подтверждено заказчиком</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Проект</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>DANIL_NAGORNIY</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>project-nagorny.html</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Дом в Тагиле 2 этажа</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Нижний Тагил</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Загородный дом</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="n">
         <v>180</v>
       </c>
-      <c r="F12" s="5" t="inlineStr"/>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Подтверждено заказчиком</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>Реализован</t>
         </is>
       </c>
-      <c r="H12" s="3" t="n">
-        <v>2025</v>
-      </c>
-      <c r="I12" s="4" t="inlineStr">
-        <is>
-          <t>A_FRAMES</t>
-        </is>
-      </c>
-      <c r="J12" s="4" t="inlineStr">
-        <is>
-          <t>project-a-frames.html</t>
-        </is>
-      </c>
-      <c r="K12" s="4" t="inlineStr"/>
-    </row>
-    <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Банный СПА-комплекс</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Свердловская обл.</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Коммерческий объект</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="n">
-        <v>190</v>
-      </c>
-      <c r="F13" s="5" t="inlineStr"/>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="H17" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>TAGIL_2_ETAGA</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>project-tagil-2-etaga.html</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Загородный дом в Тагиле</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Нижний Тагил</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Загородный дом</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>240</v>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Подтверждено заказчиком</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Проект</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>TAGIL_DOM</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>project-tagil-dom.html</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Дом Сергей</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Нижний Тагил</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Загородный дом</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>160</v>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Подтверждено заказчиком</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>Реализован</t>
         </is>
       </c>
-      <c r="H13" s="3" t="n">
-        <v>2025</v>
-      </c>
-      <c r="I13" s="4" t="inlineStr">
-        <is>
-          <t>BANNIY_KOMPL</t>
-        </is>
-      </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>project-banniy-kompl.html</t>
-        </is>
-      </c>
-      <c r="K13" s="4" t="inlineStr"/>
-    </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="3" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Частная резиденция ХМАО</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Сургут / ХМАО</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>Загородный дом</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="n">
-        <v>340</v>
-      </c>
-      <c r="F14" s="5" t="inlineStr"/>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>Проект</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="n">
-        <v>2026</v>
-      </c>
-      <c r="I14" s="4" t="inlineStr">
-        <is>
-          <t>HMAO</t>
-        </is>
-      </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>project-hmao.html</t>
-        </is>
-      </c>
-      <c r="K14" s="4" t="inlineStr"/>
-    </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Апартаменты в Сочи</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Сочи</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>Жилая квартира</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="n">
-        <v>90</v>
-      </c>
-      <c r="F15" s="5" t="inlineStr"/>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>Реализован</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="n">
-        <v>2025</v>
-      </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>SOCHI_KVARTIRA</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>project-sochi-kvartira.html</t>
-        </is>
-      </c>
-      <c r="K15" s="4" t="inlineStr"/>
-    </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Коттедж Данил Нагорный</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Свердловская обл.</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Загородный дом</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="n">
-        <v>180</v>
-      </c>
-      <c r="F16" s="5" t="inlineStr"/>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>Проект</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="n">
-        <v>2025</v>
-      </c>
-      <c r="I16" s="4" t="inlineStr">
-        <is>
-          <t>DANIL_NAGORNIY</t>
-        </is>
-      </c>
-      <c r="J16" s="4" t="inlineStr">
-        <is>
-          <t>project-nagorny.html</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr"/>
-    </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Дом в Тагиле 2 этажа</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Нижний Тагил</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Загородный дом</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="n">
-        <v>240</v>
-      </c>
-      <c r="F17" s="5" t="inlineStr"/>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>Реализован</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="n">
+      <c r="H19" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t>TAGIL_2_ETAGA</t>
-        </is>
-      </c>
-      <c r="J17" s="4" t="inlineStr">
-        <is>
-          <t>project-tagil-2-etaga.html</t>
-        </is>
-      </c>
-      <c r="K17" s="4" t="inlineStr"/>
-    </row>
-    <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="3" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Загородный дом в Тагиле</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Нижний Тагил</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Загородный дом</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="n">
-        <v>210</v>
-      </c>
-      <c r="F18" s="5" t="inlineStr"/>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>Проект</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="n">
-        <v>2024</v>
-      </c>
-      <c r="I18" s="4" t="inlineStr">
-        <is>
-          <t>TAGIL_DOM</t>
-        </is>
-      </c>
-      <c r="J18" s="4" t="inlineStr">
-        <is>
-          <t>project-tagil-dom.html</t>
-        </is>
-      </c>
-      <c r="K18" s="4" t="inlineStr"/>
-    </row>
-    <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="3" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Дом Сергей</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Нижний Тагил</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Загородный дом</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="F19" s="5" t="inlineStr"/>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>Реализован</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="n">
-        <v>2024</v>
-      </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="I19" s="3" t="inlineStr">
         <is>
           <t>TAGIL_SERGEY</t>
         </is>
       </c>
-      <c r="J19" s="4" t="inlineStr">
+      <c r="J19" s="3" t="inlineStr">
         <is>
           <t>project-sergey.html</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr"/>
+      <c r="K19" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>